<commit_message>
Stadium and Orion Manufacturing BOMs updated as per issue #12
</commit_message>
<xml_diff>
--- a/Deliverables/Orion_Board/BOM/Manufacturer-BOM-Orion.xlsx
+++ b/Deliverables/Orion_Board/BOM/Manufacturer-BOM-Orion.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24729"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\SH-CircuitCorrections\Deliverables\Orion_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\SH-CircuitCorrections\Deliverables\Orion_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD8B5A2-EC01-44C9-BA87-04B1696862A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9795"/>
+    <workbookView xWindow="7710" yWindow="0" windowWidth="10335" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="75">
   <si>
     <t>S. No.</t>
   </si>
@@ -220,17 +221,38 @@
     <t>AP2310</t>
   </si>
   <si>
-    <t xml:space="preserve">HoAR0805-1/8W-10KR-0.1%-TCR25
+    <t>Out of Stock on LCSC</t>
+  </si>
+  <si>
+    <t>Chipmall</t>
+  </si>
+  <si>
+    <t>Not available on LCSC</t>
+  </si>
+  <si>
+    <t>Arrow</t>
+  </si>
+  <si>
+    <t>Not available on LCSC. Orignal part out of stock.</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>Out of Stock on LCSC. Similar not available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0805W8F1002T5E
 </t>
   </si>
   <si>
-    <t>Out of Stock on LCSC</t>
+    <t>Orignal part is out of Stock on LCSC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -581,7 +603,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -597,9 +619,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -627,9 +646,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -684,95 +700,110 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1049,7 +1080,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
@@ -1057,19 +1088,19 @@
     <col min="2" max="2" width="30.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" thickBot="1">
       <c r="A2" s="2" t="s">
@@ -1092,535 +1123,541 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A3" s="43">
+      <c r="A3" s="38">
         <v>1</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="22">
+      <c r="D3" s="20">
         <v>2</v>
       </c>
-      <c r="E3" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="51"/>
-    </row>
-    <row r="4" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A4" s="43">
+      <c r="E3" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="46"/>
+    </row>
+    <row r="4" spans="1:6" ht="30.75" thickBot="1">
+      <c r="A4" s="38">
         <v>2</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="14">
         <v>1</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="52" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="7" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A5" s="44">
+      <c r="E4" s="7"/>
+      <c r="F4" s="61" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="6" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A5" s="39">
         <v>3</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="14">
         <v>3</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="53"/>
+      <c r="E5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="48"/>
     </row>
     <row r="6" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A6" s="43">
+      <c r="A6" s="38">
         <v>4</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="14">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="54"/>
-    </row>
-    <row r="7" spans="1:6" s="9" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A7" s="43">
+      <c r="E6" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="49"/>
+    </row>
+    <row r="7" spans="1:6" s="8" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A7" s="38">
         <v>5</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <v>2</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="54"/>
+      <c r="E7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="49"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A8" s="43">
+      <c r="A8" s="38">
         <v>6</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="64" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <v>2</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="54"/>
+      <c r="E8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="49"/>
     </row>
     <row r="9" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A9" s="43">
+      <c r="A9" s="38">
         <v>7</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="65" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="24">
+      <c r="D9" s="22">
         <v>2</v>
       </c>
-      <c r="E9" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="55" t="s">
+      <c r="E9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="50" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A10" s="43">
+      <c r="A10" s="38">
         <v>8</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="20">
         <v>1</v>
       </c>
-      <c r="E10" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="51"/>
+      <c r="E10" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="46"/>
     </row>
     <row r="11" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A11" s="43">
+      <c r="A11" s="38">
         <v>9</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="22">
         <v>2</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="55" t="s">
-        <v>67</v>
+      <c r="E11" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="50" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A12" s="43">
+      <c r="A12" s="38">
         <v>10</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="38" t="s">
+      <c r="C12" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="25">
         <v>1</v>
       </c>
-      <c r="E12" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="56" t="s">
+      <c r="E12" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="51" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A13" s="43">
+      <c r="A13" s="38">
         <v>11</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="25">
         <v>1</v>
       </c>
-      <c r="E13" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="57"/>
+      <c r="E13" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="52"/>
     </row>
     <row r="14" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A14" s="43">
+      <c r="A14" s="38">
         <v>12</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="66" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="39">
+      <c r="D14" s="34">
         <v>3</v>
       </c>
-      <c r="E14" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="56" t="s">
+      <c r="E14" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="51" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A15" s="43">
+    <row r="15" spans="1:6" ht="30.75" thickBot="1">
+      <c r="A15" s="38">
         <v>13</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="20">
         <v>4</v>
       </c>
-      <c r="E15" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F15" s="51"/>
+      <c r="E15" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="61" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A16" s="43">
+      <c r="A16" s="38">
         <v>14</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="14">
         <v>1</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F16" s="54"/>
-    </row>
-    <row r="17" spans="1:6" s="9" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A17" s="43">
+      <c r="E16" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" spans="1:6" s="8" customFormat="1" ht="26.25" thickBot="1">
+      <c r="A17" s="38">
         <v>15</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="32">
+        <v>9</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="53" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="6" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A18" s="38">
+        <v>16</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="14">
+        <v>2</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="48"/>
+    </row>
+    <row r="19" spans="1:6" s="8" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A19" s="38">
+        <v>17</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="14">
+        <v>2</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="49"/>
+    </row>
+    <row r="20" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A20" s="38">
+        <v>18</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="22">
+        <v>2</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="54"/>
+    </row>
+    <row r="21" spans="1:6" s="6" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A21" s="43">
+        <v>19</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="27">
+        <v>5</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="55"/>
+    </row>
+    <row r="22" spans="1:6" ht="16.5" thickBot="1">
+      <c r="A22" s="38">
+        <v>20</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="29">
+        <v>1</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="46"/>
+    </row>
+    <row r="23" spans="1:6" s="8" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A23" s="38">
+        <v>21</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" s="10">
+        <v>1</v>
+      </c>
+      <c r="E23" s="63"/>
+      <c r="F23" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="35">
-        <v>9</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F17" s="58" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="7" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A18" s="43">
-        <v>16</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="16">
-        <v>2</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="53"/>
-    </row>
-    <row r="19" spans="1:6" s="9" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A19" s="43">
-        <v>17</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="16">
-        <v>2</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="54"/>
-    </row>
-    <row r="20" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A20" s="43">
-        <v>18</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="24">
-        <v>2</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F20" s="59"/>
-    </row>
-    <row r="21" spans="1:6" s="7" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A21" s="48">
-        <v>19</v>
-      </c>
-      <c r="B21" s="46" t="s">
-        <v>33</v>
-      </c>
-      <c r="C21" s="46" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="29">
-        <v>5</v>
-      </c>
-      <c r="E21" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="60"/>
-    </row>
-    <row r="22" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A22" s="43">
-        <v>20</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="31">
-        <v>1</v>
-      </c>
-      <c r="E22" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="51"/>
-    </row>
-    <row r="23" spans="1:6" s="9" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A23" s="43">
-        <v>21</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D23" s="11">
-        <v>1</v>
-      </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="52" t="s">
-        <v>67</v>
-      </c>
     </row>
     <row r="24" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A24" s="43">
+      <c r="A24" s="38">
         <v>22</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>58</v>
       </c>
       <c r="D24" s="3">
         <v>1</v>
       </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="58" t="s">
-        <v>67</v>
-      </c>
+      <c r="E24" s="62" t="s">
+        <v>71</v>
+      </c>
+      <c r="F24" s="53"/>
     </row>
     <row r="25" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A25" s="43">
+      <c r="A25" s="38">
         <v>23</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D25" s="3">
         <v>2</v>
       </c>
-      <c r="E25" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F25" s="61"/>
+      <c r="E25" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" s="56"/>
     </row>
     <row r="26" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A26" s="45">
+      <c r="A26" s="40">
         <v>24</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="D26" s="49">
+      <c r="D26" s="44">
         <v>1</v>
       </c>
-      <c r="E26" s="50" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" s="62"/>
+      <c r="E26" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="57"/>
     </row>
     <row r="27" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A27" s="43">
+      <c r="A27" s="38">
         <v>25</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="29">
         <v>1</v>
       </c>
-      <c r="E27" s="32"/>
-      <c r="F27" s="63" t="s">
+      <c r="E27" s="30" t="s">
         <v>67</v>
       </c>
+      <c r="F27" s="58" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A28" s="43">
+      <c r="A28" s="38">
         <v>26</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D28" s="3">
         <v>1</v>
       </c>
-      <c r="E28" s="18"/>
-      <c r="F28" s="52" t="s">
-        <v>67</v>
+      <c r="E28" s="16"/>
+      <c r="F28" s="47" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A29" s="43">
+      <c r="A29" s="38">
         <v>27</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>49</v>
       </c>
       <c r="D29" s="3">
         <v>1</v>
       </c>
-      <c r="E29" s="18"/>
-      <c r="F29" s="52" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A30" s="43">
+      <c r="E29" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="47" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="30.75" thickBot="1">
+      <c r="A30" s="38">
         <v>28</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D30" s="3">
         <v>1</v>
       </c>
-      <c r="E30" s="19"/>
-      <c r="F30" s="52" t="s">
-        <v>67</v>
+      <c r="E30" s="17"/>
+      <c r="F30" s="61" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="16.5" thickBot="1">
-      <c r="A31" s="43">
+      <c r="A31" s="38">
         <v>29</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="30">
+      <c r="D31" s="28">
         <v>1</v>
       </c>
-      <c r="E31" s="33"/>
-      <c r="F31" s="55" t="s">
-        <v>67</v>
+      <c r="E31" s="31"/>
+      <c r="F31" s="50" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1676,29 +1713,32 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="E26" r:id="rId1"/>
-    <hyperlink ref="E22" r:id="rId2"/>
-    <hyperlink ref="E21" r:id="rId3"/>
-    <hyperlink ref="E16" r:id="rId4"/>
-    <hyperlink ref="E11" r:id="rId5"/>
-    <hyperlink ref="E10" r:id="rId6"/>
-    <hyperlink ref="E20" r:id="rId7"/>
-    <hyperlink ref="E19" r:id="rId8"/>
-    <hyperlink ref="E18" r:id="rId9"/>
-    <hyperlink ref="E15" r:id="rId10"/>
-    <hyperlink ref="E8" r:id="rId11"/>
-    <hyperlink ref="E3" r:id="rId12"/>
-    <hyperlink ref="E7" r:id="rId13"/>
-    <hyperlink ref="E6" r:id="rId14"/>
-    <hyperlink ref="E5" r:id="rId15"/>
-    <hyperlink ref="E25" r:id="rId16"/>
-    <hyperlink ref="E9" r:id="rId17"/>
-    <hyperlink ref="E12" r:id="rId18"/>
-    <hyperlink ref="E13" r:id="rId19"/>
-    <hyperlink ref="E14" r:id="rId20"/>
-    <hyperlink ref="E17" r:id="rId21"/>
+    <hyperlink ref="E26" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E22" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E21" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E16" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E11" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E20" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E19" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="E15" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E8" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E3" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E7" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E6" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E5" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E9" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E12" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E13" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E14" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E17" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E27" r:id="rId22" xr:uid="{5D3D1099-20B3-4E60-9E24-F6048E91C53E}"/>
+    <hyperlink ref="E29" r:id="rId23" xr:uid="{7FB0C8CC-4D1F-4DFE-874E-77DCEAE2D852}"/>
+    <hyperlink ref="E24" r:id="rId24" xr:uid="{8F485E83-0E95-498A-B907-52D0C8F49D87}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>